<commit_message>
Update logistics and RE developer demos with prospect-branded deliverables
Logistics: OSM Worldwide-branded cash flow, AR aging, budget vs actual, monthly financials
RE Developer: Tangent Development-branded pro forma, draw package, investor report
Regenerated preview PNGs for all updated files

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/demos/logistics/ar-aging.xlsx
+++ b/public/demos/logistics/ar-aging.xlsx
@@ -12,11 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection Actions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="TotalAR">'AR Aging Detail'!$G$14</definedName>
-    <definedName name="TotalRetainage">'AR Aging Detail'!$H$14</definedName>
-    <definedName name="GrandTotalAR">'AR Aging Detail'!$I$14</definedName>
-    <definedName name="WeightedDSO">'AR Aging Detail'!$K$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AR Aging Detail'!$A$6:$R$13</definedName>
+    <definedName name="TotalAR">'AR Aging Detail'!$G$19</definedName>
+    <definedName name="TotalRetainage">'AR Aging Detail'!$H$19</definedName>
+    <definedName name="GrandTotalAR">'AR Aging Detail'!$I$19</definedName>
+    <definedName name="WeightedDSO">'AR Aging Detail'!$K$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AR Aging Detail'!$A$6:$R$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'AR Aging Detail'!$1:$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -680,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -706,7 +706,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Acme Construction LLC</t>
+          <t>OSM Worldwide</t>
         </is>
       </c>
     </row>
@@ -776,14 +776,14 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Retainage
-Receivable</t>
+          <t>Credit Memos
+Pending</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Total Incl.
-Retainage</t>
+Credits</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -843,56 +843,56 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Metro Development Group</t>
+          <t>Pacific Coast DTC Brands</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>210000</v>
+        <v>1850000</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>145000</v>
+        <v>420000</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>110000</v>
+        <v>0</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>85000</v>
+        <v>0</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>62000</v>
+        <v>0</v>
       </c>
       <c r="G7" s="8">
         <f>SUM(B7:F7)</f>
         <v/>
       </c>
       <c r="H7" s="7" t="n">
-        <v>70500</v>
+        <v>0</v>
       </c>
       <c r="I7" s="8">
         <f>G7+H7</f>
         <v/>
       </c>
       <c r="J7" s="9" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>94.3</v>
+        <v>34.2</v>
       </c>
       <c r="L7" s="11">
         <f>K7-J7</f>
         <v/>
       </c>
       <c r="M7" s="12">
-        <f>IF(I$14=0,0,I7/I$14)</f>
+        <f>IF(I$19=0,0,I7/I$19)</f>
         <v/>
       </c>
       <c r="N7" s="13" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/22/2026</t>
         </is>
       </c>
       <c r="O7" s="7" t="n">
-        <v>50000</v>
+        <v>1680000</v>
       </c>
       <c r="P7" s="14">
         <f>IF(N7="","",TODAY()-N7)</f>
@@ -900,7 +900,7 @@
       </c>
       <c r="Q7" s="15" t="inlineStr">
         <is>
-          <t>CRITICAL: 120+ balance growing. Owner meeting scheduled 4/5. Withholding final retainage release until current.</t>
+          <t>Largest account. eCommerce beauty/wellness brands. Pays consistently within terms. Q1 volume up 15%.</t>
         </is>
       </c>
       <c r="R7" s="16">
@@ -911,17 +911,17 @@
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Westfield School District</t>
+          <t>Midwest Fulfillment Co</t>
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>185000</v>
+        <v>1420000</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>92000</v>
+        <v>680000</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>0</v>
+        <v>125000</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>0</v>
@@ -934,7 +934,7 @@
         <v/>
       </c>
       <c r="H8" s="18" t="n">
-        <v>94500</v>
+        <v>0</v>
       </c>
       <c r="I8" s="19">
         <f>G8+H8</f>
@@ -944,23 +944,23 @@
         <v>30</v>
       </c>
       <c r="K8" s="21" t="n">
-        <v>38.2</v>
+        <v>42.8</v>
       </c>
       <c r="L8" s="22">
         <f>K8-J8</f>
         <v/>
       </c>
       <c r="M8" s="23">
-        <f>IF(I$14=0,0,I8/I$14)</f>
+        <f>IF(I$19=0,0,I8/I$19)</f>
         <v/>
       </c>
       <c r="N8" s="24" t="inlineStr">
         <is>
-          <t>03/15/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="O8" s="18" t="n">
-        <v>210000</v>
+        <v>950000</v>
       </c>
       <c r="P8" s="25">
         <f>IF(N8="","",TODAY()-N8)</f>
@@ -968,7 +968,7 @@
       </c>
       <c r="Q8" s="26" t="inlineStr">
         <is>
-          <t>Reliable payer. Processing through district AP. No concerns.</t>
+          <t>61-90 balance is disputed surcharge from January ($125K). Billing team reviewing. Customer otherwise reliable.</t>
         </is>
       </c>
       <c r="R8" s="27">
@@ -979,20 +979,20 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Greenfield Logistics Inc</t>
+          <t>National Home Goods Direct</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>310000</v>
+        <v>1150000</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0</v>
+        <v>520000</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0</v>
+        <v>280000</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0</v>
+        <v>145000</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>0</v>
@@ -1002,33 +1002,33 @@
         <v/>
       </c>
       <c r="H9" s="7" t="n">
-        <v>31000</v>
+        <v>0</v>
       </c>
       <c r="I9" s="8">
         <f>G9+H9</f>
         <v/>
       </c>
       <c r="J9" s="9" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>55.2</v>
+        <v>58.3</v>
       </c>
       <c r="L9" s="11">
         <f>K9-J9</f>
         <v/>
       </c>
       <c r="M9" s="12">
-        <f>IF(I$14=0,0,I9/I$14)</f>
+        <f>IF(I$19=0,0,I9/I$19)</f>
         <v/>
       </c>
       <c r="N9" s="13" t="inlineStr">
         <is>
-          <t>03/18/2026</t>
+          <t>02/28/2026</t>
         </is>
       </c>
       <c r="O9" s="7" t="n">
-        <v>310000</v>
+        <v>420000</v>
       </c>
       <c r="P9" s="14">
         <f>IF(N9="","",TODAY()-N9)</f>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="Q9" s="15" t="inlineStr">
         <is>
-          <t>New client, first project. NET 60 terms. Paying on schedule.</t>
+          <t>WATCH: DSO trending up. NET 45 terms but averaging 58 days. 91-120 balance includes holiday peak overage dispute ($145K). CFO call scheduled 4/10.</t>
         </is>
       </c>
       <c r="R9" s="16">
@@ -1047,17 +1047,17 @@
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
         <is>
-          <t>Riverside Health Partners</t>
+          <t>East Coast Beauty Brands</t>
         </is>
       </c>
       <c r="B10" s="18" t="n">
-        <v>125000</v>
+        <v>980000</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>68000</v>
+        <v>310000</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>45000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>0</v>
@@ -1070,7 +1070,7 @@
         <v/>
       </c>
       <c r="H10" s="18" t="n">
-        <v>79000</v>
+        <v>0</v>
       </c>
       <c r="I10" s="19">
         <f>G10+H10</f>
@@ -1080,23 +1080,23 @@
         <v>30</v>
       </c>
       <c r="K10" s="21" t="n">
-        <v>52.7</v>
+        <v>36.5</v>
       </c>
       <c r="L10" s="22">
         <f>K10-J10</f>
         <v/>
       </c>
       <c r="M10" s="23">
-        <f>IF(I$14=0,0,I10/I$14)</f>
+        <f>IF(I$19=0,0,I10/I$19)</f>
         <v/>
       </c>
       <c r="N10" s="24" t="inlineStr">
         <is>
-          <t>02/28/2026</t>
+          <t>03/18/2026</t>
         </is>
       </c>
       <c r="O10" s="18" t="n">
-        <v>95000</v>
+        <v>890000</v>
       </c>
       <c r="P10" s="25">
         <f>IF(N10="","",TODAY()-N10)</f>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="Q10" s="26" t="inlineStr">
         <is>
-          <t>61-90 bucket is disputed CO #3 ($45K). PM escalated to owner 3/20.</t>
+          <t>Strong payer. Ramping volume through York PA facility. 31-60 is normal billing cycle timing.</t>
         </is>
       </c>
       <c r="R10" s="27">
@@ -1115,17 +1115,17 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Summit Brewing Co</t>
+          <t>Other Customers (12 accounts)</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>0</v>
+        <v>910000</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>35000</v>
+        <v>280000</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
@@ -1138,7 +1138,7 @@
         <v/>
       </c>
       <c r="H11" s="7" t="n">
-        <v>49700</v>
+        <v>0</v>
       </c>
       <c r="I11" s="8">
         <f>G11+H11</f>
@@ -1148,23 +1148,23 @@
         <v>30</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>67.8</v>
+        <v>35</v>
       </c>
       <c r="L11" s="11">
         <f>K11-J11</f>
         <v/>
       </c>
       <c r="M11" s="12">
-        <f>IF(I$14=0,0,I11/I$14)</f>
+        <f>IF(I$19=0,0,I11/I$19)</f>
         <v/>
       </c>
       <c r="N11" s="13" t="inlineStr">
         <is>
-          <t>02/14/2026</t>
+          <t>03/28/2026</t>
         </is>
       </c>
       <c r="O11" s="7" t="n">
-        <v>45000</v>
+        <v>850000</v>
       </c>
       <c r="P11" s="14">
         <f>IF(N11="","",TODAY()-N11)</f>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="Q11" s="15" t="inlineStr">
         <is>
-          <t>Slow payer. 61-90 balance is Feb billing. Called 3/25, promised payment by 4/10.</t>
+          <t>Aggregated small accounts. All current or within normal billing cycles. No collection concerns.</t>
         </is>
       </c>
       <c r="R11" s="16">
@@ -1183,17 +1183,17 @@
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
         <is>
-          <t>Township of Oakdale</t>
+          <t>UrbanBox Subscription Co</t>
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>48000</v>
+        <v>680000</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>0</v>
+        <v>340000</v>
       </c>
       <c r="D12" s="18" t="n">
-        <v>0</v>
+        <v>165000</v>
       </c>
       <c r="E12" s="18" t="n">
         <v>0</v>
@@ -1206,7 +1206,7 @@
         <v/>
       </c>
       <c r="H12" s="18" t="n">
-        <v>56250</v>
+        <v>0</v>
       </c>
       <c r="I12" s="19">
         <f>G12+H12</f>
@@ -1216,23 +1216,23 @@
         <v>30</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>28.5</v>
+        <v>48.7</v>
       </c>
       <c r="L12" s="22">
         <f>K12-J12</f>
         <v/>
       </c>
       <c r="M12" s="23">
-        <f>IF(I$14=0,0,I12/I$14)</f>
+        <f>IF(I$19=0,0,I12/I$19)</f>
         <v/>
       </c>
       <c r="N12" s="24" t="inlineStr">
         <is>
-          <t>03/22/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="O12" s="18" t="n">
-        <v>125000</v>
+        <v>520000</v>
       </c>
       <c r="P12" s="25">
         <f>IF(N12="","",TODAY()-N12)</f>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="Q12" s="26" t="inlineStr">
         <is>
-          <t>Municipal client. Always pays within terms. Near project completion.</t>
+          <t>Subscription box company. Cash flow driven by subscriber cycles. 61-90 balance is Feb billing — expects payment by 4/15.</t>
         </is>
       </c>
       <c r="R12" s="27">
@@ -1251,14 +1251,14 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Harbor Point Partners LLC</t>
+          <t>SunBelt eCommerce Group</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>0</v>
+        <v>820000</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>42000</v>
+        <v>195000</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>0</v>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="H13" s="7" t="n">
-        <v>19750</v>
+        <v>0</v>
       </c>
       <c r="I13" s="8">
         <f>G13+H13</f>
@@ -1284,23 +1284,23 @@
         <v>30</v>
       </c>
       <c r="K13" s="10" t="n">
-        <v>44.1</v>
+        <v>33.1</v>
       </c>
       <c r="L13" s="11">
         <f>K13-J13</f>
         <v/>
       </c>
       <c r="M13" s="12">
-        <f>IF(I$14=0,0,I13/I$14)</f>
+        <f>IF(I$19=0,0,I13/I$19)</f>
         <v/>
       </c>
       <c r="N13" s="13" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>03/25/2026</t>
         </is>
       </c>
       <c r="O13" s="7" t="n">
-        <v>65000</v>
+        <v>780000</v>
       </c>
       <c r="P13" s="14">
         <f>IF(N13="","",TODAY()-N13)</f>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="Q13" s="15" t="inlineStr">
         <is>
-          <t>Standard payer. 31-60 is March billing in normal cycle.</t>
+          <t>Dallas facility primary shipper. Reliable NET 30 payer. Growing account — added pet supplies vertical in March.</t>
         </is>
       </c>
       <c r="R13" s="16">
@@ -1317,83 +1317,423 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Heritage Apparel Group</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>520000</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>260000</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="19">
+        <f>SUM(B14:F14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="19">
+        <f>G14+H14</f>
+        <v/>
+      </c>
+      <c r="J14" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="K14" s="21" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="L14" s="22">
+        <f>K14-J14</f>
+        <v/>
+      </c>
+      <c r="M14" s="23">
+        <f>IF(I$19=0,0,I14/I$19)</f>
+        <v/>
+      </c>
+      <c r="N14" s="24" t="inlineStr">
+        <is>
+          <t>03/15/2026</t>
+        </is>
+      </c>
+      <c r="O14" s="18" t="n">
+        <v>480000</v>
+      </c>
+      <c r="P14" s="25">
+        <f>IF(N14="","",TODAY()-N14)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="26" t="inlineStr">
+        <is>
+          <t>Fashion/apparel DTC. Multi-facility shipper (Atlanta + York PA). Solid payment history.</t>
+        </is>
+      </c>
+      <c r="R14" s="27">
+        <f>IF(F14&gt;0,"CRITICAL",IF(E14&gt;0,"HIGH",IF(D14&gt;0,"MEDIUM","")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Great Lakes Pet Supply</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>450000</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>120000</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="8">
+        <f>SUM(B15:F15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="8">
+        <f>G15+H15</f>
+        <v/>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="K15" s="10" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="L15" s="11">
+        <f>K15-J15</f>
+        <v/>
+      </c>
+      <c r="M15" s="12">
+        <f>IF(I$19=0,0,I15/I$19)</f>
+        <v/>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>03/20/2026</t>
+        </is>
+      </c>
+      <c r="O15" s="7" t="n">
+        <v>410000</v>
+      </c>
+      <c r="P15" s="14">
+        <f>IF(N15="","",TODAY()-N15)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="15" t="inlineStr">
+        <is>
+          <t>Chicago facility. Pet food/supplies. Consistent payer, seasonal volume peaks in spring and holiday.</t>
+        </is>
+      </c>
+      <c r="R15" s="16">
+        <f>IF(F15&gt;0,"CRITICAL",IF(E15&gt;0,"HIGH",IF(D15&gt;0,"MEDIUM","")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Velocity Sports Direct</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>350000</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>68000</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="19">
+        <f>SUM(B16:F16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="19">
+        <f>G16+H16</f>
+        <v/>
+      </c>
+      <c r="J16" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="K16" s="21" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="L16" s="22">
+        <f>K16-J16</f>
+        <v/>
+      </c>
+      <c r="M16" s="23">
+        <f>IF(I$19=0,0,I16/I$19)</f>
+        <v/>
+      </c>
+      <c r="N16" s="24" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="O16" s="18" t="n">
+        <v>320000</v>
+      </c>
+      <c r="P16" s="25">
+        <f>IF(N16="","",TODAY()-N16)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="26" t="inlineStr">
+        <is>
+          <t>Sporting goods. 61-90 balance tied to return processing credit dispute ($68K). Resolution expected by mid-April.</t>
+        </is>
+      </c>
+      <c r="R16" s="27">
+        <f>IF(F16&gt;0,"CRITICAL",IF(E16&gt;0,"HIGH",IF(D16&gt;0,"MEDIUM","")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>FreshDirect Supplements</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>290000</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>85000</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>42000</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>28000</v>
+      </c>
+      <c r="G17" s="8">
+        <f>SUM(B17:F17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="8">
+        <f>G17+H17</f>
+        <v/>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="K17" s="10" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="L17" s="11">
+        <f>K17-J17</f>
+        <v/>
+      </c>
+      <c r="M17" s="12">
+        <f>IF(I$19=0,0,I17/I$19)</f>
+        <v/>
+      </c>
+      <c r="N17" s="13" t="inlineStr">
+        <is>
+          <t>02/14/2026</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="n">
+        <v>180000</v>
+      </c>
+      <c r="P17" s="14">
+        <f>IF(N17="","",TODAY()-N17)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="15" t="inlineStr">
+        <is>
+          <t>CONCERN: 120+ balance ($28K) from November. Claims product was damaged in transit. Insurance claim filed. Collection call weekly until resolved.</t>
+        </is>
+      </c>
+      <c r="R17" s="16">
+        <f>IF(F17&gt;0,"CRITICAL",IF(E17&gt;0,"HIGH",IF(D17&gt;0,"MEDIUM","")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>TechGear Outlet</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n">
+        <v>380000</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="19">
+        <f>SUM(B18:F18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="19">
+        <f>G18+H18</f>
+        <v/>
+      </c>
+      <c r="J18" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="K18" s="21" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="L18" s="22">
+        <f>K18-J18</f>
+        <v/>
+      </c>
+      <c r="M18" s="23">
+        <f>IF(I$19=0,0,I18/I$19)</f>
+        <v/>
+      </c>
+      <c r="N18" s="24" t="inlineStr">
+        <is>
+          <t>03/28/2026</t>
+        </is>
+      </c>
+      <c r="O18" s="18" t="n">
+        <v>365000</v>
+      </c>
+      <c r="P18" s="25">
+        <f>IF(N18="","",TODAY()-N18)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="26" t="inlineStr">
+        <is>
+          <t>Consumer electronics. Fast payer — often pays within 25 days. High-value parcels, insured shipments.</t>
+        </is>
+      </c>
+      <c r="R18" s="27">
+        <f>IF(F18&gt;0,"CRITICAL",IF(E18&gt;0,"HIGH",IF(D18&gt;0,"MEDIUM","")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B14" s="29">
-        <f>SUM(B7:B13)</f>
-        <v/>
-      </c>
-      <c r="C14" s="29">
-        <f>SUM(C7:C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="29">
-        <f>SUM(D7:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="29">
-        <f>SUM(E7:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="29">
-        <f>SUM(F7:F13)</f>
-        <v/>
-      </c>
-      <c r="G14" s="29">
-        <f>SUM(G7:G13)</f>
-        <v/>
-      </c>
-      <c r="H14" s="29">
-        <f>SUM(H7:H13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="29">
-        <f>SUM(I7:I13)</f>
-        <v/>
-      </c>
-      <c r="J14" s="30" t="n"/>
-      <c r="K14" s="31">
-        <f>IF(G14=0,0,SUMPRODUCT(K7:K13,G7:G13)/G14)</f>
-        <v/>
-      </c>
-      <c r="L14" s="31">
-        <f>IF(G14=0,0,SUMPRODUCT(L7:L13,G7:G13)/G14)</f>
-        <v/>
-      </c>
-      <c r="M14" s="30" t="n"/>
-      <c r="N14" s="30" t="n"/>
-      <c r="O14" s="30" t="n"/>
-      <c r="P14" s="30" t="n"/>
-      <c r="Q14" s="30" t="n"/>
-      <c r="R14" s="30" t="n"/>
+      <c r="B19" s="29">
+        <f>SUM(B7:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="29">
+        <f>SUM(C7:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="29">
+        <f>SUM(D7:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="29">
+        <f>SUM(E7:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="29">
+        <f>SUM(F7:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="29">
+        <f>SUM(G7:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="29">
+        <f>SUM(H7:H18)</f>
+        <v/>
+      </c>
+      <c r="I19" s="29">
+        <f>SUM(I7:I18)</f>
+        <v/>
+      </c>
+      <c r="J19" s="30" t="n"/>
+      <c r="K19" s="31">
+        <f>IF(G19=0,0,SUMPRODUCT(K7:K18,G7:G18)/G19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="31">
+        <f>IF(G19=0,0,SUMPRODUCT(L7:L18,G7:G18)/G19)</f>
+        <v/>
+      </c>
+      <c r="M19" s="30" t="n"/>
+      <c r="N19" s="30" t="n"/>
+      <c r="O19" s="30" t="n"/>
+      <c r="P19" s="30" t="n"/>
+      <c r="Q19" s="30" t="n"/>
+      <c r="R19" s="30" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A6:R13"/>
+  <autoFilter ref="A6:R18"/>
   <mergeCells count="4">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="F7:F13">
+  <conditionalFormatting sqref="F7:F18">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E7:E13">
+  <conditionalFormatting sqref="E7:E18">
     <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D7:D13">
+  <conditionalFormatting sqref="D7:D18">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M7:M13">
+  <conditionalFormatting sqref="M7:M18">
     <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="2">
       <formula>0.25</formula>
     </cfRule>
@@ -1401,7 +1741,7 @@
       <formula>AND(M7&gt;0.15,M7&lt;=0.25)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L7:L13">
+  <conditionalFormatting sqref="L7:L18">
     <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
       <formula>30</formula>
     </cfRule>
@@ -1409,7 +1749,7 @@
       <formula>15</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P7:P13">
+  <conditionalFormatting sqref="P7:P18">
     <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="0">
       <formula>90</formula>
     </cfRule>
@@ -1450,7 +1790,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Acme Construction LLC</t>
+          <t>OSM Worldwide</t>
         </is>
       </c>
     </row>
@@ -1483,29 +1823,29 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>'AR Aging Detail'!G14</f>
+        <f>'AR Aging Detail'!G19</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="33" t="inlineStr">
         <is>
-          <t>Total Retainage Receivable</t>
+          <t>Credit Memos Pending</t>
         </is>
       </c>
       <c r="B7" s="8">
-        <f>'AR Aging Detail'!H14</f>
+        <f>'AR Aging Detail'!H19</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="33" t="inlineStr">
         <is>
-          <t>Grand Total Receivable</t>
+          <t>Grand Total Receivable (incl. Credits)</t>
         </is>
       </c>
       <c r="B8" s="8">
-        <f>'AR Aging Detail'!I14</f>
+        <f>'AR Aging Detail'!I19</f>
         <v/>
       </c>
     </row>
@@ -1516,7 +1856,7 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!B14/'AR Aging Detail'!G14)</f>
+        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!B19/'AR Aging Detail'!G19)</f>
         <v/>
       </c>
     </row>
@@ -1527,7 +1867,7 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!C14/'AR Aging Detail'!G14)</f>
+        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!C19/'AR Aging Detail'!G19)</f>
         <v/>
       </c>
     </row>
@@ -1538,7 +1878,7 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!D14/'AR Aging Detail'!G14)</f>
+        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!D19/'AR Aging Detail'!G19)</f>
         <v/>
       </c>
     </row>
@@ -1549,7 +1889,7 @@
         </is>
       </c>
       <c r="B12" s="12">
-        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!E14/'AR Aging Detail'!G14)</f>
+        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!E19/'AR Aging Detail'!G19)</f>
         <v/>
       </c>
     </row>
@@ -1560,7 +1900,7 @@
         </is>
       </c>
       <c r="B13" s="12">
-        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!F14/'AR Aging Detail'!G14)</f>
+        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!F19/'AR Aging Detail'!G19)</f>
         <v/>
       </c>
     </row>
@@ -1571,7 +1911,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>'AR Aging Detail'!K14</f>
+        <f>'AR Aging Detail'!K19</f>
         <v/>
       </c>
     </row>
@@ -1582,7 +1922,7 @@
         </is>
       </c>
       <c r="B15" s="34">
-        <f>INDEX('AR Aging Detail'!A:A,MATCH(MAX('AR Aging Detail'!I7:I13),'AR Aging Detail'!I7:I13,0))</f>
+        <f>INDEX('AR Aging Detail'!A:A,MATCH(MAX('AR Aging Detail'!I7:I18),'AR Aging Detail'!I7:I18,0))</f>
         <v/>
       </c>
     </row>
@@ -1593,7 +1933,7 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>MAX('AR Aging Detail'!M7:M13)</f>
+        <f>MAX('AR Aging Detail'!M7:M18)</f>
         <v/>
       </c>
     </row>
@@ -1604,7 +1944,7 @@
         </is>
       </c>
       <c r="B17" s="8">
-        <f>SUM('AR Aging Detail'!C14:'AR Aging Detail'!F14)</f>
+        <f>SUM('AR Aging Detail'!C19:'AR Aging Detail'!F19)</f>
         <v/>
       </c>
     </row>
@@ -1615,7 +1955,7 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>IF('AR Aging Detail'!G14=0,0,(SUM('AR Aging Detail'!C14:'AR Aging Detail'!F14))/'AR Aging Detail'!G14)</f>
+        <f>IF('AR Aging Detail'!G19=0,0,(SUM('AR Aging Detail'!C19:'AR Aging Detail'!F19))/'AR Aging Detail'!G19)</f>
         <v/>
       </c>
     </row>
@@ -1626,7 +1966,7 @@
         </is>
       </c>
       <c r="B19" s="8">
-        <f>'AR Aging Detail'!D14*0.05+'AR Aging Detail'!E14*0.10+'AR Aging Detail'!F14*0.25</f>
+        <f>'AR Aging Detail'!D19*0.05+'AR Aging Detail'!E19*0.10+'AR Aging Detail'!F19*0.25</f>
         <v/>
       </c>
     </row>
@@ -1644,7 +1984,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>1875000</v>
+        <v>13900000</v>
       </c>
     </row>
     <row r="23">
@@ -1654,7 +1994,7 @@
         </is>
       </c>
       <c r="B23" s="35">
-        <f>'AR Aging Detail'!G14-B22</f>
+        <f>'AR Aging Detail'!G19-B22</f>
         <v/>
       </c>
     </row>
@@ -1710,16 +2050,16 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>1620000</v>
+        <v>12100000</v>
       </c>
       <c r="C28" s="36" t="n">
-        <v>0.55</v>
+        <v>0.62</v>
       </c>
       <c r="D28" s="36" t="n">
-        <v>0.45</v>
+        <v>0.38</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>48.2</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="29">
@@ -1729,16 +2069,16 @@
         </is>
       </c>
       <c r="B29" s="18" t="n">
-        <v>1710000</v>
+        <v>13200000</v>
       </c>
       <c r="C29" s="37" t="n">
-        <v>0.52</v>
+        <v>0.58</v>
       </c>
       <c r="D29" s="37" t="n">
-        <v>0.48</v>
+        <v>0.42</v>
       </c>
       <c r="E29" s="21" t="n">
-        <v>51</v>
+        <v>40.2</v>
       </c>
     </row>
     <row r="30">
@@ -1748,16 +2088,16 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>1540000</v>
+        <v>14500000</v>
       </c>
       <c r="C30" s="36" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="36" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>44.8</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="31">
@@ -1767,16 +2107,16 @@
         </is>
       </c>
       <c r="B31" s="18" t="n">
-        <v>1850000</v>
+        <v>13500000</v>
       </c>
       <c r="C31" s="37" t="n">
-        <v>0.48</v>
+        <v>0.6</v>
       </c>
       <c r="D31" s="37" t="n">
-        <v>0.52</v>
+        <v>0.4</v>
       </c>
       <c r="E31" s="21" t="n">
-        <v>55.3</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="32">
@@ -1786,16 +2126,16 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>1875000</v>
+        <v>13900000</v>
       </c>
       <c r="C32" s="36" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="D32" s="36" t="n">
-        <v>0.5</v>
+        <v>0.42</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>52.1</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="33">
@@ -1805,19 +2145,19 @@
         </is>
       </c>
       <c r="B33" s="19">
-        <f>'AR Aging Detail'!G14</f>
+        <f>'AR Aging Detail'!G19</f>
         <v/>
       </c>
       <c r="C33" s="23">
-        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!B14/'AR Aging Detail'!G14)</f>
+        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!B19/'AR Aging Detail'!G19)</f>
         <v/>
       </c>
       <c r="D33" s="23">
-        <f>IF('AR Aging Detail'!G14=0,0,SUM('AR Aging Detail'!C14:'AR Aging Detail'!F14)/'AR Aging Detail'!G14)</f>
+        <f>IF('AR Aging Detail'!G19=0,0,SUM('AR Aging Detail'!C19:'AR Aging Detail'!F19)/'AR Aging Detail'!G19)</f>
         <v/>
       </c>
       <c r="E33" s="22">
-        <f>'AR Aging Detail'!K14</f>
+        <f>'AR Aging Detail'!K19</f>
         <v/>
       </c>
     </row>
@@ -1839,7 +2179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1858,7 +2198,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Acme Construction LLC</t>
+          <t>OSM Worldwide</t>
         </is>
       </c>
     </row>
@@ -1944,11 +2284,11 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Metro Development Group</t>
+          <t>FreshDirect Supplements</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>257000</v>
+        <v>70000</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -1960,17 +2300,17 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>James Holloway</t>
+          <t>Chris Martinez</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>jholloway@metrodev.com / (555) 456-7890</t>
+          <t>cmartinez@freshdirectsupps.com / (305) 555-2345</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>CRITICAL: 120+ balance growing. Owner meeting scheduled 4/5. Withholding final retainage release until current.</t>
+          <t>CONCERN: 120+ balance ($28K) from November. Claims product was damaged in transit. Insurance claim filed. Collection call weekly until resolved.</t>
         </is>
       </c>
       <c r="I6" s="39" t="inlineStr">
@@ -1983,42 +2323,42 @@
     </row>
     <row r="7">
       <c r="A7" s="41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Riverside Health Partners</t>
+          <t>National Home Goods Direct</t>
         </is>
       </c>
       <c r="C7" s="19" t="n">
-        <v>45000</v>
+        <v>425000</v>
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>61-90 days</t>
+          <t>91-120 days</t>
         </is>
       </c>
       <c r="E7" s="25" t="n">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>David Park</t>
+          <t>Robert Flynn</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>dpark@riversidehealth.com / (555) 345-6789</t>
+          <t>rflynn@nationalhomegoods.com / (404) 555-3456</t>
         </is>
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t>61-90 bucket is disputed CO #3 ($45K). PM escalated to owner 3/20.</t>
+          <t>WATCH: DSO trending up. NET 45 terms but averaging 58 days. 91-120 balance includes holiday peak overage dispute ($145K). CFO call scheduled 4/10.</t>
         </is>
       </c>
       <c r="I7" s="42" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>Demand Letter</t>
         </is>
       </c>
       <c r="J7" s="17" t="n"/>
@@ -2030,11 +2370,11 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Summit Brewing Co</t>
+          <t>UrbanBox Subscription Co</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>28000</v>
+        <v>165000</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -2046,17 +2386,17 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Tom Brennan</t>
+          <t>Derek Williams</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>tbrennan@summitbrewing.com / (555) 890-1234</t>
+          <t>dwilliams@urbanbox.com / (702) 555-4567</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Slow payer. 61-90 balance is Feb billing. Called 3/25, promised payment by 4/10.</t>
+          <t>Subscription box company. Cash flow driven by subscriber cycles. 61-90 balance is Feb billing — expects payment by 4/15.</t>
         </is>
       </c>
       <c r="I8" s="39" t="inlineStr">
@@ -2066,6 +2406,92 @@
       </c>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="40" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Midwest Fulfillment Co</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>125000</v>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>61-90 days</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>75</v>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>Jason Keller</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="inlineStr">
+        <is>
+          <t>jkeller@midwestfulfill.com / (312) 555-2345</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>61-90 balance is disputed surcharge from January ($125K). Billing team reviewing. Customer otherwise reliable.</t>
+        </is>
+      </c>
+      <c r="I9" s="42" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="n"/>
+      <c r="K9" s="43" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Velocity Sports Direct</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>68000</v>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>61-90 days</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Mike Thompson</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>mthompson@velocitysports.com / (480) 555-6789</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Sporting goods. 61-90 balance tied to return processing credit dispute ($68K). Resolution expected by mid-April.</t>
+        </is>
+      </c>
+      <c r="I10" s="39" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="40" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2073,7 +2499,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:A8">
+  <conditionalFormatting sqref="A6:A10">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>1</formula>
     </cfRule>

</xml_diff>

<commit_message>
Revert logistics and RE developer demos to generic mock data
Website demos must use generic company names (not prospect-specific) since
any prospect in the industry can access the demo page URL.
Prospect-branded files are sent directly via email, not hosted publicly.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/demos/logistics/ar-aging.xlsx
+++ b/public/demos/logistics/ar-aging.xlsx
@@ -12,11 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection Actions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="TotalAR">'AR Aging Detail'!$G$19</definedName>
-    <definedName name="TotalRetainage">'AR Aging Detail'!$H$19</definedName>
-    <definedName name="GrandTotalAR">'AR Aging Detail'!$I$19</definedName>
-    <definedName name="WeightedDSO">'AR Aging Detail'!$K$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AR Aging Detail'!$A$6:$R$18</definedName>
+    <definedName name="TotalAR">'AR Aging Detail'!$G$14</definedName>
+    <definedName name="TotalRetainage">'AR Aging Detail'!$H$14</definedName>
+    <definedName name="GrandTotalAR">'AR Aging Detail'!$I$14</definedName>
+    <definedName name="WeightedDSO">'AR Aging Detail'!$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AR Aging Detail'!$A$6:$R$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'AR Aging Detail'!$1:$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -680,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -706,7 +706,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OSM Worldwide</t>
+          <t>Acme Construction LLC</t>
         </is>
       </c>
     </row>
@@ -776,14 +776,14 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Credit Memos
-Pending</t>
+          <t>Retainage
+Receivable</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Total Incl.
-Credits</t>
+Retainage</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -843,56 +843,56 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Pacific Coast DTC Brands</t>
+          <t>Metro Development Group</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>1850000</v>
+        <v>210000</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>420000</v>
+        <v>145000</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0</v>
+        <v>110000</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>0</v>
+        <v>62000</v>
       </c>
       <c r="G7" s="8">
         <f>SUM(B7:F7)</f>
         <v/>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0</v>
+        <v>70500</v>
       </c>
       <c r="I7" s="8">
         <f>G7+H7</f>
         <v/>
       </c>
       <c r="J7" s="9" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>34.2</v>
+        <v>94.3</v>
       </c>
       <c r="L7" s="11">
         <f>K7-J7</f>
         <v/>
       </c>
       <c r="M7" s="12">
-        <f>IF(I$19=0,0,I7/I$19)</f>
+        <f>IF(I$14=0,0,I7/I$14)</f>
         <v/>
       </c>
       <c r="N7" s="13" t="inlineStr">
         <is>
-          <t>03/22/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="O7" s="7" t="n">
-        <v>1680000</v>
+        <v>50000</v>
       </c>
       <c r="P7" s="14">
         <f>IF(N7="","",TODAY()-N7)</f>
@@ -900,7 +900,7 @@
       </c>
       <c r="Q7" s="15" t="inlineStr">
         <is>
-          <t>Largest account. eCommerce beauty/wellness brands. Pays consistently within terms. Q1 volume up 15%.</t>
+          <t>CRITICAL: 120+ balance growing. Owner meeting scheduled 4/5. Withholding final retainage release until current.</t>
         </is>
       </c>
       <c r="R7" s="16">
@@ -911,17 +911,17 @@
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Midwest Fulfillment Co</t>
+          <t>Westfield School District</t>
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>1420000</v>
+        <v>185000</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>680000</v>
+        <v>92000</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>125000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>0</v>
@@ -934,7 +934,7 @@
         <v/>
       </c>
       <c r="H8" s="18" t="n">
-        <v>0</v>
+        <v>94500</v>
       </c>
       <c r="I8" s="19">
         <f>G8+H8</f>
@@ -944,23 +944,23 @@
         <v>30</v>
       </c>
       <c r="K8" s="21" t="n">
-        <v>42.8</v>
+        <v>38.2</v>
       </c>
       <c r="L8" s="22">
         <f>K8-J8</f>
         <v/>
       </c>
       <c r="M8" s="23">
-        <f>IF(I$19=0,0,I8/I$19)</f>
+        <f>IF(I$14=0,0,I8/I$14)</f>
         <v/>
       </c>
       <c r="N8" s="24" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>03/15/2026</t>
         </is>
       </c>
       <c r="O8" s="18" t="n">
-        <v>950000</v>
+        <v>210000</v>
       </c>
       <c r="P8" s="25">
         <f>IF(N8="","",TODAY()-N8)</f>
@@ -968,7 +968,7 @@
       </c>
       <c r="Q8" s="26" t="inlineStr">
         <is>
-          <t>61-90 balance is disputed surcharge from January ($125K). Billing team reviewing. Customer otherwise reliable.</t>
+          <t>Reliable payer. Processing through district AP. No concerns.</t>
         </is>
       </c>
       <c r="R8" s="27">
@@ -979,20 +979,20 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>National Home Goods Direct</t>
+          <t>Greenfield Logistics Inc</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>1150000</v>
+        <v>310000</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>520000</v>
+        <v>0</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>280000</v>
+        <v>0</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>145000</v>
+        <v>0</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>0</v>
@@ -1002,33 +1002,33 @@
         <v/>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0</v>
+        <v>31000</v>
       </c>
       <c r="I9" s="8">
         <f>G9+H9</f>
         <v/>
       </c>
       <c r="J9" s="9" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>58.3</v>
+        <v>55.2</v>
       </c>
       <c r="L9" s="11">
         <f>K9-J9</f>
         <v/>
       </c>
       <c r="M9" s="12">
-        <f>IF(I$19=0,0,I9/I$19)</f>
+        <f>IF(I$14=0,0,I9/I$14)</f>
         <v/>
       </c>
       <c r="N9" s="13" t="inlineStr">
         <is>
-          <t>02/28/2026</t>
+          <t>03/18/2026</t>
         </is>
       </c>
       <c r="O9" s="7" t="n">
-        <v>420000</v>
+        <v>310000</v>
       </c>
       <c r="P9" s="14">
         <f>IF(N9="","",TODAY()-N9)</f>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="Q9" s="15" t="inlineStr">
         <is>
-          <t>WATCH: DSO trending up. NET 45 terms but averaging 58 days. 91-120 balance includes holiday peak overage dispute ($145K). CFO call scheduled 4/10.</t>
+          <t>New client, first project. NET 60 terms. Paying on schedule.</t>
         </is>
       </c>
       <c r="R9" s="16">
@@ -1047,17 +1047,17 @@
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
         <is>
-          <t>East Coast Beauty Brands</t>
+          <t>Riverside Health Partners</t>
         </is>
       </c>
       <c r="B10" s="18" t="n">
-        <v>980000</v>
+        <v>125000</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>310000</v>
+        <v>68000</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>0</v>
+        <v>45000</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>0</v>
@@ -1070,7 +1070,7 @@
         <v/>
       </c>
       <c r="H10" s="18" t="n">
-        <v>0</v>
+        <v>79000</v>
       </c>
       <c r="I10" s="19">
         <f>G10+H10</f>
@@ -1080,23 +1080,23 @@
         <v>30</v>
       </c>
       <c r="K10" s="21" t="n">
-        <v>36.5</v>
+        <v>52.7</v>
       </c>
       <c r="L10" s="22">
         <f>K10-J10</f>
         <v/>
       </c>
       <c r="M10" s="23">
-        <f>IF(I$19=0,0,I10/I$19)</f>
+        <f>IF(I$14=0,0,I10/I$14)</f>
         <v/>
       </c>
       <c r="N10" s="24" t="inlineStr">
         <is>
-          <t>03/18/2026</t>
+          <t>02/28/2026</t>
         </is>
       </c>
       <c r="O10" s="18" t="n">
-        <v>890000</v>
+        <v>95000</v>
       </c>
       <c r="P10" s="25">
         <f>IF(N10="","",TODAY()-N10)</f>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="Q10" s="26" t="inlineStr">
         <is>
-          <t>Strong payer. Ramping volume through York PA facility. 31-60 is normal billing cycle timing.</t>
+          <t>61-90 bucket is disputed CO #3 ($45K). PM escalated to owner 3/20.</t>
         </is>
       </c>
       <c r="R10" s="27">
@@ -1115,17 +1115,17 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Other Customers (12 accounts)</t>
+          <t>Summit Brewing Co</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>910000</v>
+        <v>0</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>280000</v>
+        <v>35000</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>0</v>
+        <v>28000</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
@@ -1138,7 +1138,7 @@
         <v/>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0</v>
+        <v>49700</v>
       </c>
       <c r="I11" s="8">
         <f>G11+H11</f>
@@ -1148,23 +1148,23 @@
         <v>30</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>35</v>
+        <v>67.8</v>
       </c>
       <c r="L11" s="11">
         <f>K11-J11</f>
         <v/>
       </c>
       <c r="M11" s="12">
-        <f>IF(I$19=0,0,I11/I$19)</f>
+        <f>IF(I$14=0,0,I11/I$14)</f>
         <v/>
       </c>
       <c r="N11" s="13" t="inlineStr">
         <is>
-          <t>03/28/2026</t>
+          <t>02/14/2026</t>
         </is>
       </c>
       <c r="O11" s="7" t="n">
-        <v>850000</v>
+        <v>45000</v>
       </c>
       <c r="P11" s="14">
         <f>IF(N11="","",TODAY()-N11)</f>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="Q11" s="15" t="inlineStr">
         <is>
-          <t>Aggregated small accounts. All current or within normal billing cycles. No collection concerns.</t>
+          <t>Slow payer. 61-90 balance is Feb billing. Called 3/25, promised payment by 4/10.</t>
         </is>
       </c>
       <c r="R11" s="16">
@@ -1183,17 +1183,17 @@
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
         <is>
-          <t>UrbanBox Subscription Co</t>
+          <t>Township of Oakdale</t>
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>680000</v>
+        <v>48000</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>340000</v>
+        <v>0</v>
       </c>
       <c r="D12" s="18" t="n">
-        <v>165000</v>
+        <v>0</v>
       </c>
       <c r="E12" s="18" t="n">
         <v>0</v>
@@ -1206,7 +1206,7 @@
         <v/>
       </c>
       <c r="H12" s="18" t="n">
-        <v>0</v>
+        <v>56250</v>
       </c>
       <c r="I12" s="19">
         <f>G12+H12</f>
@@ -1216,23 +1216,23 @@
         <v>30</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>48.7</v>
+        <v>28.5</v>
       </c>
       <c r="L12" s="22">
         <f>K12-J12</f>
         <v/>
       </c>
       <c r="M12" s="23">
-        <f>IF(I$19=0,0,I12/I$19)</f>
+        <f>IF(I$14=0,0,I12/I$14)</f>
         <v/>
       </c>
       <c r="N12" s="24" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>03/22/2026</t>
         </is>
       </c>
       <c r="O12" s="18" t="n">
-        <v>520000</v>
+        <v>125000</v>
       </c>
       <c r="P12" s="25">
         <f>IF(N12="","",TODAY()-N12)</f>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="Q12" s="26" t="inlineStr">
         <is>
-          <t>Subscription box company. Cash flow driven by subscriber cycles. 61-90 balance is Feb billing — expects payment by 4/15.</t>
+          <t>Municipal client. Always pays within terms. Near project completion.</t>
         </is>
       </c>
       <c r="R12" s="27">
@@ -1251,14 +1251,14 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>SunBelt eCommerce Group</t>
+          <t>Harbor Point Partners LLC</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>820000</v>
+        <v>0</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>195000</v>
+        <v>42000</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>0</v>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0</v>
+        <v>19750</v>
       </c>
       <c r="I13" s="8">
         <f>G13+H13</f>
@@ -1284,23 +1284,23 @@
         <v>30</v>
       </c>
       <c r="K13" s="10" t="n">
-        <v>33.1</v>
+        <v>44.1</v>
       </c>
       <c r="L13" s="11">
         <f>K13-J13</f>
         <v/>
       </c>
       <c r="M13" s="12">
-        <f>IF(I$19=0,0,I13/I$19)</f>
+        <f>IF(I$14=0,0,I13/I$14)</f>
         <v/>
       </c>
       <c r="N13" s="13" t="inlineStr">
         <is>
-          <t>03/25/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="O13" s="7" t="n">
-        <v>780000</v>
+        <v>65000</v>
       </c>
       <c r="P13" s="14">
         <f>IF(N13="","",TODAY()-N13)</f>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="Q13" s="15" t="inlineStr">
         <is>
-          <t>Dallas facility primary shipper. Reliable NET 30 payer. Growing account — added pet supplies vertical in March.</t>
+          <t>Standard payer. 31-60 is March billing in normal cycle.</t>
         </is>
       </c>
       <c r="R13" s="16">
@@ -1317,423 +1317,83 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t>Heritage Apparel Group</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="n">
-        <v>520000</v>
-      </c>
-      <c r="C14" s="18" t="n">
-        <v>260000</v>
-      </c>
-      <c r="D14" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="19">
-        <f>SUM(B14:F14)</f>
-        <v/>
-      </c>
-      <c r="H14" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="19">
-        <f>G14+H14</f>
-        <v/>
-      </c>
-      <c r="J14" s="20" t="n">
-        <v>30</v>
-      </c>
-      <c r="K14" s="21" t="n">
-        <v>37.9</v>
-      </c>
-      <c r="L14" s="22">
-        <f>K14-J14</f>
-        <v/>
-      </c>
-      <c r="M14" s="23">
-        <f>IF(I$19=0,0,I14/I$19)</f>
-        <v/>
-      </c>
-      <c r="N14" s="24" t="inlineStr">
-        <is>
-          <t>03/15/2026</t>
-        </is>
-      </c>
-      <c r="O14" s="18" t="n">
-        <v>480000</v>
-      </c>
-      <c r="P14" s="25">
-        <f>IF(N14="","",TODAY()-N14)</f>
-        <v/>
-      </c>
-      <c r="Q14" s="26" t="inlineStr">
-        <is>
-          <t>Fashion/apparel DTC. Multi-facility shipper (Atlanta + York PA). Solid payment history.</t>
-        </is>
-      </c>
-      <c r="R14" s="27">
-        <f>IF(F14&gt;0,"CRITICAL",IF(E14&gt;0,"HIGH",IF(D14&gt;0,"MEDIUM","")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Great Lakes Pet Supply</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>450000</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>120000</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="8">
-        <f>SUM(B15:F15)</f>
-        <v/>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="8">
-        <f>G15+H15</f>
-        <v/>
-      </c>
-      <c r="J15" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="K15" s="10" t="n">
-        <v>31.8</v>
-      </c>
-      <c r="L15" s="11">
-        <f>K15-J15</f>
-        <v/>
-      </c>
-      <c r="M15" s="12">
-        <f>IF(I$19=0,0,I15/I$19)</f>
-        <v/>
-      </c>
-      <c r="N15" s="13" t="inlineStr">
-        <is>
-          <t>03/20/2026</t>
-        </is>
-      </c>
-      <c r="O15" s="7" t="n">
-        <v>410000</v>
-      </c>
-      <c r="P15" s="14">
-        <f>IF(N15="","",TODAY()-N15)</f>
-        <v/>
-      </c>
-      <c r="Q15" s="15" t="inlineStr">
-        <is>
-          <t>Chicago facility. Pet food/supplies. Consistent payer, seasonal volume peaks in spring and holiday.</t>
-        </is>
-      </c>
-      <c r="R15" s="16">
-        <f>IF(F15&gt;0,"CRITICAL",IF(E15&gt;0,"HIGH",IF(D15&gt;0,"MEDIUM","")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Velocity Sports Direct</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="n">
-        <v>350000</v>
-      </c>
-      <c r="C16" s="18" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D16" s="18" t="n">
-        <v>68000</v>
-      </c>
-      <c r="E16" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="19">
-        <f>SUM(B16:F16)</f>
-        <v/>
-      </c>
-      <c r="H16" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="19">
-        <f>G16+H16</f>
-        <v/>
-      </c>
-      <c r="J16" s="20" t="n">
-        <v>30</v>
-      </c>
-      <c r="K16" s="21" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="L16" s="22">
-        <f>K16-J16</f>
-        <v/>
-      </c>
-      <c r="M16" s="23">
-        <f>IF(I$19=0,0,I16/I$19)</f>
-        <v/>
-      </c>
-      <c r="N16" s="24" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="O16" s="18" t="n">
-        <v>320000</v>
-      </c>
-      <c r="P16" s="25">
-        <f>IF(N16="","",TODAY()-N16)</f>
-        <v/>
-      </c>
-      <c r="Q16" s="26" t="inlineStr">
-        <is>
-          <t>Sporting goods. 61-90 balance tied to return processing credit dispute ($68K). Resolution expected by mid-April.</t>
-        </is>
-      </c>
-      <c r="R16" s="27">
-        <f>IF(F16&gt;0,"CRITICAL",IF(E16&gt;0,"HIGH",IF(D16&gt;0,"MEDIUM","")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>FreshDirect Supplements</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>290000</v>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>85000</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>42000</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>28000</v>
-      </c>
-      <c r="G17" s="8">
-        <f>SUM(B17:F17)</f>
-        <v/>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="8">
-        <f>G17+H17</f>
-        <v/>
-      </c>
-      <c r="J17" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="K17" s="10" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="L17" s="11">
-        <f>K17-J17</f>
-        <v/>
-      </c>
-      <c r="M17" s="12">
-        <f>IF(I$19=0,0,I17/I$19)</f>
-        <v/>
-      </c>
-      <c r="N17" s="13" t="inlineStr">
-        <is>
-          <t>02/14/2026</t>
-        </is>
-      </c>
-      <c r="O17" s="7" t="n">
-        <v>180000</v>
-      </c>
-      <c r="P17" s="14">
-        <f>IF(N17="","",TODAY()-N17)</f>
-        <v/>
-      </c>
-      <c r="Q17" s="15" t="inlineStr">
-        <is>
-          <t>CONCERN: 120+ balance ($28K) from November. Claims product was damaged in transit. Insurance claim filed. Collection call weekly until resolved.</t>
-        </is>
-      </c>
-      <c r="R17" s="16">
-        <f>IF(F17&gt;0,"CRITICAL",IF(E17&gt;0,"HIGH",IF(D17&gt;0,"MEDIUM","")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>TechGear Outlet</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="n">
-        <v>380000</v>
-      </c>
-      <c r="C18" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="19">
-        <f>SUM(B18:F18)</f>
-        <v/>
-      </c>
-      <c r="H18" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="19">
-        <f>G18+H18</f>
-        <v/>
-      </c>
-      <c r="J18" s="20" t="n">
-        <v>30</v>
-      </c>
-      <c r="K18" s="21" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="L18" s="22">
-        <f>K18-J18</f>
-        <v/>
-      </c>
-      <c r="M18" s="23">
-        <f>IF(I$19=0,0,I18/I$19)</f>
-        <v/>
-      </c>
-      <c r="N18" s="24" t="inlineStr">
-        <is>
-          <t>03/28/2026</t>
-        </is>
-      </c>
-      <c r="O18" s="18" t="n">
-        <v>365000</v>
-      </c>
-      <c r="P18" s="25">
-        <f>IF(N18="","",TODAY()-N18)</f>
-        <v/>
-      </c>
-      <c r="Q18" s="26" t="inlineStr">
-        <is>
-          <t>Consumer electronics. Fast payer — often pays within 25 days. High-value parcels, insured shipments.</t>
-        </is>
-      </c>
-      <c r="R18" s="27">
-        <f>IF(F18&gt;0,"CRITICAL",IF(E18&gt;0,"HIGH",IF(D18&gt;0,"MEDIUM","")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B19" s="29">
-        <f>SUM(B7:B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="29">
-        <f>SUM(C7:C18)</f>
-        <v/>
-      </c>
-      <c r="D19" s="29">
-        <f>SUM(D7:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="29">
-        <f>SUM(E7:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="29">
-        <f>SUM(F7:F18)</f>
-        <v/>
-      </c>
-      <c r="G19" s="29">
-        <f>SUM(G7:G18)</f>
-        <v/>
-      </c>
-      <c r="H19" s="29">
-        <f>SUM(H7:H18)</f>
-        <v/>
-      </c>
-      <c r="I19" s="29">
-        <f>SUM(I7:I18)</f>
-        <v/>
-      </c>
-      <c r="J19" s="30" t="n"/>
-      <c r="K19" s="31">
-        <f>IF(G19=0,0,SUMPRODUCT(K7:K18,G7:G18)/G19)</f>
-        <v/>
-      </c>
-      <c r="L19" s="31">
-        <f>IF(G19=0,0,SUMPRODUCT(L7:L18,G7:G18)/G19)</f>
-        <v/>
-      </c>
-      <c r="M19" s="30" t="n"/>
-      <c r="N19" s="30" t="n"/>
-      <c r="O19" s="30" t="n"/>
-      <c r="P19" s="30" t="n"/>
-      <c r="Q19" s="30" t="n"/>
-      <c r="R19" s="30" t="n"/>
+      <c r="B14" s="29">
+        <f>SUM(B7:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="29">
+        <f>SUM(C7:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="29">
+        <f>SUM(D7:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="29">
+        <f>SUM(E7:E13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="29">
+        <f>SUM(F7:F13)</f>
+        <v/>
+      </c>
+      <c r="G14" s="29">
+        <f>SUM(G7:G13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="29">
+        <f>SUM(H7:H13)</f>
+        <v/>
+      </c>
+      <c r="I14" s="29">
+        <f>SUM(I7:I13)</f>
+        <v/>
+      </c>
+      <c r="J14" s="30" t="n"/>
+      <c r="K14" s="31">
+        <f>IF(G14=0,0,SUMPRODUCT(K7:K13,G7:G13)/G14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="31">
+        <f>IF(G14=0,0,SUMPRODUCT(L7:L13,G7:G13)/G14)</f>
+        <v/>
+      </c>
+      <c r="M14" s="30" t="n"/>
+      <c r="N14" s="30" t="n"/>
+      <c r="O14" s="30" t="n"/>
+      <c r="P14" s="30" t="n"/>
+      <c r="Q14" s="30" t="n"/>
+      <c r="R14" s="30" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A6:R18"/>
+  <autoFilter ref="A6:R13"/>
   <mergeCells count="4">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="F7:F18">
+  <conditionalFormatting sqref="F7:F13">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E7:E18">
+  <conditionalFormatting sqref="E7:E13">
     <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D7:D18">
+  <conditionalFormatting sqref="D7:D13">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M7:M18">
+  <conditionalFormatting sqref="M7:M13">
     <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="2">
       <formula>0.25</formula>
     </cfRule>
@@ -1741,7 +1401,7 @@
       <formula>AND(M7&gt;0.15,M7&lt;=0.25)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L7:L18">
+  <conditionalFormatting sqref="L7:L13">
     <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
       <formula>30</formula>
     </cfRule>
@@ -1749,7 +1409,7 @@
       <formula>15</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P7:P18">
+  <conditionalFormatting sqref="P7:P13">
     <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="0">
       <formula>90</formula>
     </cfRule>
@@ -1790,7 +1450,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OSM Worldwide</t>
+          <t>Acme Construction LLC</t>
         </is>
       </c>
     </row>
@@ -1823,29 +1483,29 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>'AR Aging Detail'!G19</f>
+        <f>'AR Aging Detail'!G14</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="33" t="inlineStr">
         <is>
-          <t>Credit Memos Pending</t>
+          <t>Total Retainage Receivable</t>
         </is>
       </c>
       <c r="B7" s="8">
-        <f>'AR Aging Detail'!H19</f>
+        <f>'AR Aging Detail'!H14</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="33" t="inlineStr">
         <is>
-          <t>Grand Total Receivable (incl. Credits)</t>
+          <t>Grand Total Receivable</t>
         </is>
       </c>
       <c r="B8" s="8">
-        <f>'AR Aging Detail'!I19</f>
+        <f>'AR Aging Detail'!I14</f>
         <v/>
       </c>
     </row>
@@ -1856,7 +1516,7 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!B19/'AR Aging Detail'!G19)</f>
+        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!B14/'AR Aging Detail'!G14)</f>
         <v/>
       </c>
     </row>
@@ -1867,7 +1527,7 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!C19/'AR Aging Detail'!G19)</f>
+        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!C14/'AR Aging Detail'!G14)</f>
         <v/>
       </c>
     </row>
@@ -1878,7 +1538,7 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!D19/'AR Aging Detail'!G19)</f>
+        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!D14/'AR Aging Detail'!G14)</f>
         <v/>
       </c>
     </row>
@@ -1889,7 +1549,7 @@
         </is>
       </c>
       <c r="B12" s="12">
-        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!E19/'AR Aging Detail'!G19)</f>
+        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!E14/'AR Aging Detail'!G14)</f>
         <v/>
       </c>
     </row>
@@ -1900,7 +1560,7 @@
         </is>
       </c>
       <c r="B13" s="12">
-        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!F19/'AR Aging Detail'!G19)</f>
+        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!F14/'AR Aging Detail'!G14)</f>
         <v/>
       </c>
     </row>
@@ -1911,7 +1571,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>'AR Aging Detail'!K19</f>
+        <f>'AR Aging Detail'!K14</f>
         <v/>
       </c>
     </row>
@@ -1922,7 +1582,7 @@
         </is>
       </c>
       <c r="B15" s="34">
-        <f>INDEX('AR Aging Detail'!A:A,MATCH(MAX('AR Aging Detail'!I7:I18),'AR Aging Detail'!I7:I18,0))</f>
+        <f>INDEX('AR Aging Detail'!A:A,MATCH(MAX('AR Aging Detail'!I7:I13),'AR Aging Detail'!I7:I13,0))</f>
         <v/>
       </c>
     </row>
@@ -1933,7 +1593,7 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>MAX('AR Aging Detail'!M7:M18)</f>
+        <f>MAX('AR Aging Detail'!M7:M13)</f>
         <v/>
       </c>
     </row>
@@ -1944,7 +1604,7 @@
         </is>
       </c>
       <c r="B17" s="8">
-        <f>SUM('AR Aging Detail'!C19:'AR Aging Detail'!F19)</f>
+        <f>SUM('AR Aging Detail'!C14:'AR Aging Detail'!F14)</f>
         <v/>
       </c>
     </row>
@@ -1955,7 +1615,7 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>IF('AR Aging Detail'!G19=0,0,(SUM('AR Aging Detail'!C19:'AR Aging Detail'!F19))/'AR Aging Detail'!G19)</f>
+        <f>IF('AR Aging Detail'!G14=0,0,(SUM('AR Aging Detail'!C14:'AR Aging Detail'!F14))/'AR Aging Detail'!G14)</f>
         <v/>
       </c>
     </row>
@@ -1966,7 +1626,7 @@
         </is>
       </c>
       <c r="B19" s="8">
-        <f>'AR Aging Detail'!D19*0.05+'AR Aging Detail'!E19*0.10+'AR Aging Detail'!F19*0.25</f>
+        <f>'AR Aging Detail'!D14*0.05+'AR Aging Detail'!E14*0.10+'AR Aging Detail'!F14*0.25</f>
         <v/>
       </c>
     </row>
@@ -1984,7 +1644,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>13900000</v>
+        <v>1875000</v>
       </c>
     </row>
     <row r="23">
@@ -1994,7 +1654,7 @@
         </is>
       </c>
       <c r="B23" s="35">
-        <f>'AR Aging Detail'!G19-B22</f>
+        <f>'AR Aging Detail'!G14-B22</f>
         <v/>
       </c>
     </row>
@@ -2050,16 +1710,16 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>12100000</v>
+        <v>1620000</v>
       </c>
       <c r="C28" s="36" t="n">
-        <v>0.62</v>
+        <v>0.55</v>
       </c>
       <c r="D28" s="36" t="n">
-        <v>0.38</v>
+        <v>0.45</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>38.5</v>
+        <v>48.2</v>
       </c>
     </row>
     <row r="29">
@@ -2069,16 +1729,16 @@
         </is>
       </c>
       <c r="B29" s="18" t="n">
-        <v>13200000</v>
+        <v>1710000</v>
       </c>
       <c r="C29" s="37" t="n">
-        <v>0.58</v>
+        <v>0.52</v>
       </c>
       <c r="D29" s="37" t="n">
-        <v>0.42</v>
+        <v>0.48</v>
       </c>
       <c r="E29" s="21" t="n">
-        <v>40.2</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30">
@@ -2088,16 +1748,16 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>14500000</v>
+        <v>1540000</v>
       </c>
       <c r="C30" s="36" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="D30" s="36" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>43.8</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="31">
@@ -2107,16 +1767,16 @@
         </is>
       </c>
       <c r="B31" s="18" t="n">
-        <v>13500000</v>
+        <v>1850000</v>
       </c>
       <c r="C31" s="37" t="n">
-        <v>0.6</v>
+        <v>0.48</v>
       </c>
       <c r="D31" s="37" t="n">
-        <v>0.4</v>
+        <v>0.52</v>
       </c>
       <c r="E31" s="21" t="n">
-        <v>41.5</v>
+        <v>55.3</v>
       </c>
     </row>
     <row r="32">
@@ -2126,16 +1786,16 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>13900000</v>
+        <v>1875000</v>
       </c>
       <c r="C32" s="36" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="D32" s="36" t="n">
-        <v>0.42</v>
+        <v>0.5</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>42.8</v>
+        <v>52.1</v>
       </c>
     </row>
     <row r="33">
@@ -2145,19 +1805,19 @@
         </is>
       </c>
       <c r="B33" s="19">
-        <f>'AR Aging Detail'!G19</f>
+        <f>'AR Aging Detail'!G14</f>
         <v/>
       </c>
       <c r="C33" s="23">
-        <f>IF('AR Aging Detail'!G19=0,0,'AR Aging Detail'!B19/'AR Aging Detail'!G19)</f>
+        <f>IF('AR Aging Detail'!G14=0,0,'AR Aging Detail'!B14/'AR Aging Detail'!G14)</f>
         <v/>
       </c>
       <c r="D33" s="23">
-        <f>IF('AR Aging Detail'!G19=0,0,SUM('AR Aging Detail'!C19:'AR Aging Detail'!F19)/'AR Aging Detail'!G19)</f>
+        <f>IF('AR Aging Detail'!G14=0,0,SUM('AR Aging Detail'!C14:'AR Aging Detail'!F14)/'AR Aging Detail'!G14)</f>
         <v/>
       </c>
       <c r="E33" s="22">
-        <f>'AR Aging Detail'!K19</f>
+        <f>'AR Aging Detail'!K14</f>
         <v/>
       </c>
     </row>
@@ -2179,7 +1839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2198,7 +1858,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OSM Worldwide</t>
+          <t>Acme Construction LLC</t>
         </is>
       </c>
     </row>
@@ -2284,11 +1944,11 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>FreshDirect Supplements</t>
+          <t>Metro Development Group</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>70000</v>
+        <v>257000</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -2300,17 +1960,17 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Chris Martinez</t>
+          <t>James Holloway</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>cmartinez@freshdirectsupps.com / (305) 555-2345</t>
+          <t>jholloway@metrodev.com / (555) 456-7890</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>CONCERN: 120+ balance ($28K) from November. Claims product was damaged in transit. Insurance claim filed. Collection call weekly until resolved.</t>
+          <t>CRITICAL: 120+ balance growing. Owner meeting scheduled 4/5. Withholding final retainage release until current.</t>
         </is>
       </c>
       <c r="I6" s="39" t="inlineStr">
@@ -2323,42 +1983,42 @@
     </row>
     <row r="7">
       <c r="A7" s="41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>National Home Goods Direct</t>
+          <t>Riverside Health Partners</t>
         </is>
       </c>
       <c r="C7" s="19" t="n">
-        <v>425000</v>
+        <v>45000</v>
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>91-120 days</t>
+          <t>61-90 days</t>
         </is>
       </c>
       <c r="E7" s="25" t="n">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>Robert Flynn</t>
+          <t>David Park</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>rflynn@nationalhomegoods.com / (404) 555-3456</t>
+          <t>dpark@riversidehealth.com / (555) 345-6789</t>
         </is>
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t>WATCH: DSO trending up. NET 45 terms but averaging 58 days. 91-120 balance includes holiday peak overage dispute ($145K). CFO call scheduled 4/10.</t>
+          <t>61-90 bucket is disputed CO #3 ($45K). PM escalated to owner 3/20.</t>
         </is>
       </c>
       <c r="I7" s="42" t="inlineStr">
         <is>
-          <t>Demand Letter</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="J7" s="17" t="n"/>
@@ -2370,11 +2030,11 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>UrbanBox Subscription Co</t>
+          <t>Summit Brewing Co</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>165000</v>
+        <v>28000</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
@@ -2386,17 +2046,17 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Derek Williams</t>
+          <t>Tom Brennan</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>dwilliams@urbanbox.com / (702) 555-4567</t>
+          <t>tbrennan@summitbrewing.com / (555) 890-1234</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Subscription box company. Cash flow driven by subscriber cycles. 61-90 balance is Feb billing — expects payment by 4/15.</t>
+          <t>Slow payer. 61-90 balance is Feb billing. Called 3/25, promised payment by 4/10.</t>
         </is>
       </c>
       <c r="I8" s="39" t="inlineStr">
@@ -2406,92 +2066,6 @@
       </c>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="40" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="41" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>Midwest Fulfillment Co</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>125000</v>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>61-90 days</t>
-        </is>
-      </c>
-      <c r="E9" s="25" t="n">
-        <v>75</v>
-      </c>
-      <c r="F9" s="17" t="inlineStr">
-        <is>
-          <t>Jason Keller</t>
-        </is>
-      </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>jkeller@midwestfulfill.com / (312) 555-2345</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="inlineStr">
-        <is>
-          <t>61-90 balance is disputed surcharge from January ($125K). Billing team reviewing. Customer otherwise reliable.</t>
-        </is>
-      </c>
-      <c r="I9" s="42" t="inlineStr">
-        <is>
-          <t>Call</t>
-        </is>
-      </c>
-      <c r="J9" s="17" t="n"/>
-      <c r="K9" s="43" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="38" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Velocity Sports Direct</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>68000</v>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>61-90 days</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>75</v>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Mike Thompson</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>mthompson@velocitysports.com / (480) 555-6789</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>Sporting goods. 61-90 balance tied to return processing credit dispute ($68K). Resolution expected by mid-April.</t>
-        </is>
-      </c>
-      <c r="I10" s="39" t="inlineStr">
-        <is>
-          <t>Call</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="n"/>
-      <c r="K10" s="40" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2499,7 +2073,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:A10">
+  <conditionalFormatting sqref="A6:A8">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>1</formula>
     </cfRule>

</xml_diff>